<commit_message>
Add 08_main_effects_controlled.Rmd for Review Comment 2
Implement multivariate models controlling for survey location,
prior visits, and residence zone to address Reviewer Comment 2
(Round 2).

Key analyses and contents:
- Calculate cross-tabulation of MEC visits by survey location (place)
  to quantify spatial distribution differences.
- Fit parsimonious logistic regression models (glm, drop1 LRT) for
  25 cognitive map elements (m_*) with visited_ome, place, visits_count,
  and distance_zone2 as predictors.
- Fit parsimonious ordinal logistic regression models (MASS::polr)
  for 8 tourist infrastructure rankings (pnuw_*).
- Include comprehensive Markdown interpretations verifying that MEC
  visitation remains statistically non-significant (p > 0.05) across
  nearly all map features and infrastructure ranks after controlling
  for confounders.
</commit_message>
<xml_diff>
--- a/PNUW_lato_2025_informacja_OME_to_R.xlsx
+++ b/PNUW_lato_2025_informacja_OME_to_R.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uam-my.sharepoint.com/personal/kp_amu_edu_pl/Documents/nauka/2025_PNUW/PNUW_informacja_OME_2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="989" documentId="8_{037AFBCB-FC45-483C-AFD2-078DE2830EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{523251A0-D770-4A35-B85D-514F64AE484F}"/>
+  <xr:revisionPtr revIDLastSave="1005" documentId="8_{037AFBCB-FC45-483C-AFD2-078DE2830EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E2E611E-F47F-48A7-90F3-A9BB7CA1F737}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="short_colname_data" sheetId="1" r:id="rId1"/>
@@ -2546,9 +2546,177 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="159">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -2802,172 +2970,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -3018,10 +3021,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <font>
@@ -3058,102 +3058,102 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:CD251" totalsRowCount="1" headerRowDxfId="158">
   <autoFilter ref="A1:CD250" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="82">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="x_id" dataDxfId="157" totalsRowDxfId="156"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="x_id" dataDxfId="55" totalsRowDxfId="54"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="x_start_time"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="x_completion_time"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="x_email" dataDxfId="155" totalsRowDxfId="154"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="x_name" dataDxfId="153" totalsRowDxfId="152"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="survey_id" dataDxfId="151" totalsRowDxfId="150"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="place" dataDxfId="149" totalsRowDxfId="148"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="x_email" dataDxfId="157" totalsRowDxfId="156"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="x_name" dataDxfId="155" totalsRowDxfId="154"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="survey_id" dataDxfId="153" totalsRowDxfId="152"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="place" dataDxfId="151" totalsRowDxfId="150"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="completion_date"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="x_interviewer" dataDxfId="147" totalsRowDxfId="146"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="visits_count" dataDxfId="145" totalsRowDxfId="144"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="main_reason" dataDxfId="143" totalsRowDxfId="142"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="infrastructure_assessment" dataDxfId="141" totalsRowDxfId="140"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="elements_shelters" dataDxfId="139" totalsRowDxfId="138"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="elements_walktrails" dataDxfId="137" totalsRowDxfId="136"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="elements_edupaths" dataDxfId="135" totalsRowDxfId="134"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="elements_biketrails" dataDxfId="133" totalsRowDxfId="132"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="elements_horsetrails" dataDxfId="131" totalsRowDxfId="130"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="elements_viewpoints" dataDxfId="129" totalsRowDxfId="128"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="elements_parking" dataDxfId="127" totalsRowDxfId="126"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="elements_bins" dataDxfId="125" totalsRowDxfId="124"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="elements_toilets" dataDxfId="123" totalsRowDxfId="122"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="elements_food" dataDxfId="121" totalsRowDxfId="120"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="elements_infoboards" dataDxfId="119" totalsRowDxfId="118"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="elements_restspots" dataDxfId="117" totalsRowDxfId="116"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="pnuw_walktrails" dataDxfId="115" totalsRowDxfId="114"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="pnuw_edupaths" dataDxfId="113" totalsRowDxfId="112"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="pnuw_biketrails" dataDxfId="111" totalsRowDxfId="110"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="pnuw_viewpoints" dataDxfId="109" totalsRowDxfId="108"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="pnuw_parking" dataDxfId="107" totalsRowDxfId="106"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="pnuw_bins" dataDxfId="105" totalsRowDxfId="104"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="pnuw_infoboards" dataDxfId="103" totalsRowDxfId="102"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="pnuw_restspots" dataDxfId="101" totalsRowDxfId="100"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="infra_change_suggested" dataDxfId="99" totalsRowDxfId="98"/>
-    <tableColumn id="82" xr3:uid="{DF96268E-7D56-4F50-9563-4F4CDD5B3B53}" name="chan_sign_info" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="96">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="x_interviewer" dataDxfId="149" totalsRowDxfId="148"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="visits_count" dataDxfId="147" totalsRowDxfId="146"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="main_reason" dataDxfId="145" totalsRowDxfId="144"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="infrastructure_assessment" dataDxfId="143" totalsRowDxfId="142"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="elements_shelters" dataDxfId="53" totalsRowDxfId="52"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="elements_walktrails" dataDxfId="51" totalsRowDxfId="50"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="elements_edupaths" dataDxfId="49" totalsRowDxfId="48"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="elements_biketrails" dataDxfId="47" totalsRowDxfId="46"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="elements_horsetrails" dataDxfId="45" totalsRowDxfId="44"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="elements_viewpoints" dataDxfId="43" totalsRowDxfId="42"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="elements_parking" dataDxfId="41" totalsRowDxfId="40"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="elements_bins" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="elements_toilets" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="elements_food" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="elements_infoboards" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="elements_restspots" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="pnuw_walktrails" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="pnuw_edupaths" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="pnuw_biketrails" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="pnuw_viewpoints" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="pnuw_parking" dataDxfId="21" totalsRowDxfId="20"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="pnuw_bins" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="pnuw_infoboards" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="pnuw_restspots" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="infra_change_suggested" dataDxfId="141" totalsRowDxfId="140"/>
+    <tableColumn id="82" xr3:uid="{DF96268E-7D56-4F50-9563-4F4CDD5B3B53}" name="chan_sign_info" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="12">
       <totalsRowFormula>COUNTIF(OfficeForms.Table[chan_sign_info],1)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="81" xr3:uid="{AF5996F3-84AE-4C5C-9217-2ECE5D5E7C34}" name="chan_access" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="94">
+    <tableColumn id="81" xr3:uid="{AF5996F3-84AE-4C5C-9217-2ECE5D5E7C34}" name="chan_access" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="10">
       <totalsRowFormula>COUNTIF(OfficeForms.Table[chan_access],1)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="80" xr3:uid="{6C1AF5E7-F0DB-4A92-BDBA-BA165E409A29}" name="chan_trails" totalsRowFunction="custom" dataDxfId="93" totalsRowDxfId="92">
+    <tableColumn id="80" xr3:uid="{6C1AF5E7-F0DB-4A92-BDBA-BA165E409A29}" name="chan_trails" totalsRowFunction="custom" dataDxfId="9" totalsRowDxfId="8">
       <totalsRowFormula>COUNTIF(OfficeForms.Table[chan_trails],1)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="79" xr3:uid="{6FE28077-2AD8-42C3-86B0-D11B64EF7186}" name="chan_viewpoints" totalsRowFunction="custom" dataDxfId="91" totalsRowDxfId="90">
+    <tableColumn id="79" xr3:uid="{6FE28077-2AD8-42C3-86B0-D11B64EF7186}" name="chan_viewpoints" totalsRowFunction="custom" dataDxfId="7" totalsRowDxfId="6">
       <totalsRowFormula>COUNTIF(OfficeForms.Table[chan_viewpoints],1)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="78" xr3:uid="{DF618B83-F1E4-49C6-8BC1-16565917F708}" name="chan_repairs" totalsRowFunction="custom" dataDxfId="89" totalsRowDxfId="88">
+    <tableColumn id="78" xr3:uid="{DF618B83-F1E4-49C6-8BC1-16565917F708}" name="chan_repairs" totalsRowFunction="custom" dataDxfId="5" totalsRowDxfId="4">
       <totalsRowFormula>COUNTIF(OfficeForms.Table[chan_repairs],1)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="77" xr3:uid="{D82DDCFA-BB47-4D82-937D-4159EDFC9B8F}" name="chan_amenities" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="86">
+    <tableColumn id="77" xr3:uid="{D82DDCFA-BB47-4D82-937D-4159EDFC9B8F}" name="chan_amenities" totalsRowFunction="custom" dataDxfId="3" totalsRowDxfId="2">
       <totalsRowFormula>COUNTIF(OfficeForms.Table[chan_amenities],1)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="76" xr3:uid="{E47D5EF4-AFB7-4605-9D26-7444A1D8507D}" name="chan_other" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="84">
+    <tableColumn id="76" xr3:uid="{E47D5EF4-AFB7-4605-9D26-7444A1D8507D}" name="chan_other" totalsRowFunction="custom" dataDxfId="1" totalsRowDxfId="0">
       <totalsRowFormula>COUNTIF(OfficeForms.Table[chan_other],1)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="trail_decision_time" dataDxfId="83" totalsRowDxfId="82"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="visited_ome" dataDxfId="81" totalsRowDxfId="80"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="it_staff_asked" dataDxfId="79" totalsRowDxfId="78"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="it_staff_range" dataDxfId="77" totalsRowDxfId="76"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="it_staff_plan_change" dataDxfId="75" totalsRowDxfId="74"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="it_staff_what" dataDxfId="73" totalsRowDxfId="72"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="it_exhibition_asked" dataDxfId="71" totalsRowDxfId="70"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="it_exhibition_range" dataDxfId="69" totalsRowDxfId="68"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="it_exhibition_plan_change" dataDxfId="67" totalsRowDxfId="66"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="it_exhibition_what" dataDxfId="65" totalsRowDxfId="64"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="sex" dataDxfId="63" totalsRowDxfId="62"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="education" dataDxfId="61" totalsRowDxfId="60"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="age" dataDxfId="59" totalsRowDxfId="58"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="residence_town" dataDxfId="57" totalsRowDxfId="56"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="residence_county" dataDxfId="55" totalsRowDxfId="54"/>
-    <tableColumn id="75" xr3:uid="{E4F3E300-581F-43C9-8F0F-2B651A79F5B4}" name="distance_zone" dataDxfId="53" totalsRowDxfId="52"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="comment" dataDxfId="51" totalsRowDxfId="50"/>
-    <tableColumn id="50" xr3:uid="{9CC5F519-5737-41A5-9B4E-0CEEE8DB8DD0}" name="m_scale" dataDxfId="49" totalsRowDxfId="48"/>
-    <tableColumn id="51" xr3:uid="{844FEE05-9D5E-4317-AF63-ACE738D77195}" name="m_border" dataDxfId="47" totalsRowDxfId="46"/>
-    <tableColumn id="52" xr3:uid="{A6379163-D180-4C15-836A-1372894E2D65}" name="m_path_asphalt" dataDxfId="45" totalsRowDxfId="44"/>
-    <tableColumn id="53" xr3:uid="{E6DBCE21-CFE6-4700-A154-908873C7E035}" name="m_path_nature" dataDxfId="43" totalsRowDxfId="42"/>
-    <tableColumn id="54" xr3:uid="{6AACF702-2E06-457E-96BC-F54FB8651FE4}" name="m_path_other" dataDxfId="41" totalsRowDxfId="40"/>
-    <tableColumn id="55" xr3:uid="{93FA03CE-92D2-4E46-A953-6BEA032A1396}" name="m_edges_border" dataDxfId="39" totalsRowDxfId="38"/>
-    <tableColumn id="56" xr3:uid="{8E30E61E-C946-467F-9C1A-716EEE16AE41}" name="m_edges_river" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="57" xr3:uid="{B74E3225-FF14-4063-99B2-BCEF95AC9B1F}" name="m_circles_lake" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="58" xr3:uid="{E0EB2628-A142-4340-9E4C-6CE26BC006CE}" name="m_circles_meadow" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="59" xr3:uid="{9606006B-B77F-4D15-9C98-F0485DC1DD6D}" name="m_nodes_parking" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="60" xr3:uid="{A8524A61-B5AC-4BC3-A5C8-C05DEE29F011}" name="m_nodes_town" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="61" xr3:uid="{20A1B6D5-D9F6-44E4-80BD-B6CD07AF3576}" name="m_nodes_headquarters" dataDxfId="27" totalsRowDxfId="26"/>
-    <tableColumn id="62" xr3:uid="{77A7442D-7E32-4665-B637-48A8FF794CCD}" name="m_nodes_ome" dataDxfId="25" totalsRowDxfId="24"/>
-    <tableColumn id="63" xr3:uid="{0F38E494-DC05-41B1-8943-40AFC98A4F16}" name="m_landmark_tower" dataDxfId="23" totalsRowDxfId="22"/>
-    <tableColumn id="64" xr3:uid="{121368F5-84B3-43B3-BA72-BA86B4C7B24E}" name="m_landmark_shelter" dataDxfId="21" totalsRowDxfId="20"/>
-    <tableColumn id="65" xr3:uid="{10421C62-F1CD-4BF1-B525-0828462C50A9}" name="m_landmark_birdhide" dataDxfId="19" totalsRowDxfId="18"/>
-    <tableColumn id="66" xr3:uid="{1C09F1C0-DFAF-4F6D-8641-9F70068BB671}" name="m_landmark_bench" dataDxfId="17" totalsRowDxfId="16"/>
-    <tableColumn id="67" xr3:uid="{3B5C8E11-FC1A-411F-ACAE-A898A88C5D9C}" name="m_landmark_chimney" dataDxfId="15" totalsRowDxfId="14"/>
-    <tableColumn id="68" xr3:uid="{BB0D1BAA-2DAB-46BC-BAB5-09B4EB9E26F1}" name="m_landmark_bridge" dataDxfId="13" totalsRowDxfId="12"/>
-    <tableColumn id="69" xr3:uid="{26F352ED-D4E3-4440-B275-F5DF81EF07C8}" name="m_landmark_ferry" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="70" xr3:uid="{D841E551-CFBA-4B05-956A-7C8215C1074F}" name="m_landmark_pump_station" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="71" xr3:uid="{E6BDC622-BB86-4603-AE48-D3FC4DDA85B4}" name="m_landmark_info_board" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="72" xr3:uid="{D52B70A2-E1CA-4097-8730-D9D1FA52A29C}" name="m_landmark_footbridge" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="73" xr3:uid="{C31610FD-2C2B-4BA6-A8EC-76E38D64A101}" name="m_event_observation" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="74" xr3:uid="{107F738D-C3D9-43F0-9866-76C38605071D}" name="m_event_people" dataDxfId="1" totalsRowDxfId="0"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="trail_decision_time" dataDxfId="139" totalsRowDxfId="138"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="visited_ome" dataDxfId="137" totalsRowDxfId="136"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="it_staff_asked" dataDxfId="135" totalsRowDxfId="134"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="it_staff_range" dataDxfId="133" totalsRowDxfId="132"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="it_staff_plan_change" dataDxfId="131" totalsRowDxfId="130"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="it_staff_what" dataDxfId="129" totalsRowDxfId="128"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="it_exhibition_asked" dataDxfId="127" totalsRowDxfId="126"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="it_exhibition_range" dataDxfId="125" totalsRowDxfId="124"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="it_exhibition_plan_change" dataDxfId="123" totalsRowDxfId="122"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="it_exhibition_what" dataDxfId="121" totalsRowDxfId="120"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="sex" dataDxfId="119" totalsRowDxfId="118"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="education" dataDxfId="117" totalsRowDxfId="116"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="age" dataDxfId="115" totalsRowDxfId="114"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="residence_town" dataDxfId="113" totalsRowDxfId="112"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="residence_county" dataDxfId="111" totalsRowDxfId="110"/>
+    <tableColumn id="75" xr3:uid="{E4F3E300-581F-43C9-8F0F-2B651A79F5B4}" name="distance_zone" dataDxfId="109" totalsRowDxfId="108"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="comment" dataDxfId="107" totalsRowDxfId="106"/>
+    <tableColumn id="50" xr3:uid="{9CC5F519-5737-41A5-9B4E-0CEEE8DB8DD0}" name="m_scale" dataDxfId="105" totalsRowDxfId="104"/>
+    <tableColumn id="51" xr3:uid="{844FEE05-9D5E-4317-AF63-ACE738D77195}" name="m_border" dataDxfId="103" totalsRowDxfId="102"/>
+    <tableColumn id="52" xr3:uid="{A6379163-D180-4C15-836A-1372894E2D65}" name="m_path_asphalt" dataDxfId="101" totalsRowDxfId="100"/>
+    <tableColumn id="53" xr3:uid="{E6DBCE21-CFE6-4700-A154-908873C7E035}" name="m_path_nature" dataDxfId="99" totalsRowDxfId="98"/>
+    <tableColumn id="54" xr3:uid="{6AACF702-2E06-457E-96BC-F54FB8651FE4}" name="m_path_other" dataDxfId="97" totalsRowDxfId="96"/>
+    <tableColumn id="55" xr3:uid="{93FA03CE-92D2-4E46-A953-6BEA032A1396}" name="m_edges_border" dataDxfId="95" totalsRowDxfId="94"/>
+    <tableColumn id="56" xr3:uid="{8E30E61E-C946-467F-9C1A-716EEE16AE41}" name="m_edges_river" dataDxfId="93" totalsRowDxfId="92"/>
+    <tableColumn id="57" xr3:uid="{B74E3225-FF14-4063-99B2-BCEF95AC9B1F}" name="m_circles_lake" dataDxfId="91" totalsRowDxfId="90"/>
+    <tableColumn id="58" xr3:uid="{E0EB2628-A142-4340-9E4C-6CE26BC006CE}" name="m_circles_meadow" dataDxfId="89" totalsRowDxfId="88"/>
+    <tableColumn id="59" xr3:uid="{9606006B-B77F-4D15-9C98-F0485DC1DD6D}" name="m_nodes_parking" dataDxfId="87" totalsRowDxfId="86"/>
+    <tableColumn id="60" xr3:uid="{A8524A61-B5AC-4BC3-A5C8-C05DEE29F011}" name="m_nodes_town" dataDxfId="85" totalsRowDxfId="84"/>
+    <tableColumn id="61" xr3:uid="{20A1B6D5-D9F6-44E4-80BD-B6CD07AF3576}" name="m_nodes_headquarters" dataDxfId="83" totalsRowDxfId="82"/>
+    <tableColumn id="62" xr3:uid="{77A7442D-7E32-4665-B637-48A8FF794CCD}" name="m_nodes_ome" dataDxfId="81" totalsRowDxfId="80"/>
+    <tableColumn id="63" xr3:uid="{0F38E494-DC05-41B1-8943-40AFC98A4F16}" name="m_landmark_tower" dataDxfId="79" totalsRowDxfId="78"/>
+    <tableColumn id="64" xr3:uid="{121368F5-84B3-43B3-BA72-BA86B4C7B24E}" name="m_landmark_shelter" dataDxfId="77" totalsRowDxfId="76"/>
+    <tableColumn id="65" xr3:uid="{10421C62-F1CD-4BF1-B525-0828462C50A9}" name="m_landmark_birdhide" dataDxfId="75" totalsRowDxfId="74"/>
+    <tableColumn id="66" xr3:uid="{1C09F1C0-DFAF-4F6D-8641-9F70068BB671}" name="m_landmark_bench" dataDxfId="73" totalsRowDxfId="72"/>
+    <tableColumn id="67" xr3:uid="{3B5C8E11-FC1A-411F-ACAE-A898A88C5D9C}" name="m_landmark_chimney" dataDxfId="71" totalsRowDxfId="70"/>
+    <tableColumn id="68" xr3:uid="{BB0D1BAA-2DAB-46BC-BAB5-09B4EB9E26F1}" name="m_landmark_bridge" dataDxfId="69" totalsRowDxfId="68"/>
+    <tableColumn id="69" xr3:uid="{26F352ED-D4E3-4440-B275-F5DF81EF07C8}" name="m_landmark_ferry" dataDxfId="67" totalsRowDxfId="66"/>
+    <tableColumn id="70" xr3:uid="{D841E551-CFBA-4B05-956A-7C8215C1074F}" name="m_landmark_pump_station" dataDxfId="65" totalsRowDxfId="64"/>
+    <tableColumn id="71" xr3:uid="{E6BDC622-BB86-4603-AE48-D3FC4DDA85B4}" name="m_landmark_info_board" dataDxfId="63" totalsRowDxfId="62"/>
+    <tableColumn id="72" xr3:uid="{D52B70A2-E1CA-4097-8730-D9D1FA52A29C}" name="m_landmark_footbridge" dataDxfId="61" totalsRowDxfId="60"/>
+    <tableColumn id="73" xr3:uid="{C31610FD-2C2B-4BA6-A8EC-76E38D64A101}" name="m_event_observation" dataDxfId="59" totalsRowDxfId="58"/>
+    <tableColumn id="74" xr3:uid="{107F738D-C3D9-43F0-9866-76C38605071D}" name="m_event_people" dataDxfId="57" totalsRowDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3474,8 +3474,10 @@
     <col min="42" max="42" width="44.44140625" customWidth="1"/>
     <col min="43" max="43" width="20" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="35.6640625" customWidth="1"/>
-    <col min="45" max="49" width="20" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="20" customWidth="1"/>
+    <col min="45" max="45" width="20" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="20" customWidth="1"/>
+    <col min="47" max="47" width="20" bestFit="1" customWidth="1"/>
+    <col min="48" max="50" width="20" customWidth="1"/>
     <col min="51" max="51" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>